<commit_message>
update formatting of supplementary tables
</commit_message>
<xml_diff>
--- a/data/disruptors_supplementary_data_tables_s1-s5.xlsx
+++ b/data/disruptors_supplementary_data_tables_s1-s5.xlsx
@@ -2274,15 +2274,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -2304,6 +2295,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2311,95 +2311,11 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill>
           <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3765,7 +3681,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:10" s="24" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" s="24" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A8" s="24" t="s">
         <v>509</v>
       </c>
@@ -4085,7 +4001,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="18" spans="1:10" s="24" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" s="24" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A18" s="24" t="s">
         <v>515</v>
       </c>
@@ -4374,86 +4290,86 @@
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="50" t="s">
         <v>520</v>
       </c>
-      <c r="B27" s="43"/>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="43"/>
-      <c r="I27" s="43"/>
-      <c r="J27" s="43"/>
+      <c r="B27" s="50"/>
+      <c r="C27" s="50"/>
+      <c r="D27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="50"/>
+      <c r="G27" s="50"/>
+      <c r="H27" s="50"/>
+      <c r="I27" s="50"/>
+      <c r="J27" s="50"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="44" t="s">
+      <c r="A28" s="51" t="s">
         <v>521</v>
       </c>
-      <c r="B28" s="44"/>
-      <c r="C28" s="44"/>
-      <c r="D28" s="44"/>
-      <c r="E28" s="44"/>
-      <c r="F28" s="44"/>
-      <c r="G28" s="44"/>
-      <c r="H28" s="44"/>
-      <c r="I28" s="44"/>
-      <c r="J28" s="44"/>
+      <c r="B28" s="51"/>
+      <c r="C28" s="51"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="51"/>
+      <c r="G28" s="51"/>
+      <c r="H28" s="51"/>
+      <c r="I28" s="51"/>
+      <c r="J28" s="51"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="44" t="s">
+      <c r="A29" s="51" t="s">
         <v>522</v>
       </c>
-      <c r="B29" s="44"/>
-      <c r="C29" s="44"/>
-      <c r="D29" s="44"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="44"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="44"/>
-      <c r="I29" s="44"/>
-      <c r="J29" s="44"/>
+      <c r="B29" s="51"/>
+      <c r="C29" s="51"/>
+      <c r="D29" s="51"/>
+      <c r="E29" s="51"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="51"/>
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="51"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="44" t="s">
+      <c r="A30" s="51" t="s">
         <v>551</v>
       </c>
-      <c r="B30" s="44"/>
-      <c r="C30" s="44"/>
-      <c r="D30" s="44"/>
-      <c r="E30" s="44"/>
-      <c r="F30" s="44"/>
-      <c r="G30" s="44"/>
-      <c r="H30" s="44"/>
-      <c r="I30" s="44"/>
-      <c r="J30" s="44"/>
+      <c r="B30" s="51"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="51"/>
+      <c r="G30" s="51"/>
+      <c r="H30" s="51"/>
+      <c r="I30" s="51"/>
+      <c r="J30" s="51"/>
     </row>
     <row r="31" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="45" t="s">
+      <c r="A31" s="52" t="s">
         <v>550</v>
       </c>
-      <c r="B31" s="45"/>
-      <c r="C31" s="45"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="45"/>
-      <c r="G31" s="45"/>
-      <c r="H31" s="45"/>
-      <c r="I31" s="45"/>
-      <c r="J31" s="45"/>
+      <c r="B31" s="52"/>
+      <c r="C31" s="52"/>
+      <c r="D31" s="52"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="52"/>
+      <c r="G31" s="52"/>
+      <c r="H31" s="52"/>
+      <c r="I31" s="52"/>
+      <c r="J31" s="52"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A1:J1"/>
     <mergeCell ref="A27:J27"/>
     <mergeCell ref="A28:J28"/>
     <mergeCell ref="A29:J29"/>
     <mergeCell ref="A30:J30"/>
     <mergeCell ref="A31:J31"/>
-    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4513,7 +4429,7 @@
       <c r="C3" s="30" t="s">
         <v>327</v>
       </c>
-      <c r="D3" s="51" t="s">
+      <c r="D3" s="48" t="s">
         <v>327</v>
       </c>
       <c r="E3" s="30" t="s">
@@ -4530,13 +4446,13 @@
       <c r="A4" s="33" t="s">
         <v>566</v>
       </c>
-      <c r="B4" s="47">
+      <c r="B4" s="44">
         <v>0.3</v>
       </c>
       <c r="C4" s="34" t="s">
         <v>323</v>
       </c>
-      <c r="D4" s="52">
+      <c r="D4" s="49">
         <v>0.05</v>
       </c>
       <c r="E4" s="34" t="s">
@@ -4553,13 +4469,13 @@
       <c r="A5" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="48">
+      <c r="B5" s="45">
         <v>140</v>
       </c>
       <c r="C5" s="30" t="s">
         <v>320</v>
       </c>
-      <c r="D5" s="51" t="s">
+      <c r="D5" s="48" t="s">
         <v>563</v>
       </c>
       <c r="E5" s="30" t="s">
@@ -4576,7 +4492,7 @@
       <c r="A6" s="32" t="s">
         <v>315</v>
       </c>
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="47" t="s">
         <v>454</v>
       </c>
       <c r="C6" s="30" t="s">
@@ -4599,13 +4515,13 @@
       <c r="A7" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="47" t="s">
         <v>561</v>
       </c>
-      <c r="C7" s="50" t="s">
+      <c r="C7" s="47" t="s">
         <v>560</v>
       </c>
-      <c r="D7" s="51">
+      <c r="D7" s="48">
         <v>40</v>
       </c>
       <c r="E7" s="30" t="s">
@@ -4628,7 +4544,7 @@
       <c r="C8" s="30" t="s">
         <v>331</v>
       </c>
-      <c r="D8" s="51" t="s">
+      <c r="D8" s="48" t="s">
         <v>308</v>
       </c>
       <c r="E8" s="30" t="s">
@@ -4651,7 +4567,7 @@
       <c r="C9" s="30" t="s">
         <v>304</v>
       </c>
-      <c r="D9" s="51" t="s">
+      <c r="D9" s="48" t="s">
         <v>558</v>
       </c>
       <c r="E9" s="30" t="s">
@@ -4668,7 +4584,7 @@
       <c r="A10" s="30" t="s">
         <v>298</v>
       </c>
-      <c r="B10" s="46">
+      <c r="B10" s="43">
         <v>3800</v>
       </c>
       <c r="C10" s="30" t="s">
@@ -4691,7 +4607,7 @@
       <c r="A11" s="36" t="s">
         <v>294</v>
       </c>
-      <c r="B11" s="49" t="s">
+      <c r="B11" s="46" t="s">
         <v>295</v>
       </c>
       <c r="C11" s="36" t="s">
@@ -10655,6 +10571,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d7940701-fd28-48c6-89b6-2769869457dd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE3B5FF1D6D93545B0A9BE76E04A5739" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b213452e5774ccb18cdbac914376359f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af" xmlns:ns3="d7940701-fd28-48c6-89b6-2769869457dd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="94bb0651eba29840b02d7d9879aff2b0" ns2:_="" ns3:_="">
     <xsd:import namespace="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
@@ -10849,27 +10785,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F179CFA0-01D1-49C4-829E-9CD6990EDE07}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="d7940701-fd28-48c6-89b6-2769869457dd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d7940701-fd28-48c6-89b6-2769869457dd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C242F3B7-E13F-47B3-89BF-DC7F2A584373}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14D4D638-0E0C-48CA-BE88-3BE2B56E957A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10886,29 +10827,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C242F3B7-E13F-47B3-89BF-DC7F2A584373}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F179CFA0-01D1-49C4-829E-9CD6990EDE07}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="d7940701-fd28-48c6-89b6-2769869457dd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add egu26 script and plots
</commit_message>
<xml_diff>
--- a/data/disruptors_supplementary_data_tables_s1-s5.xlsx
+++ b/data/disruptors_supplementary_data_tables_s1-s5.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="168" documentId="8_{2185ED28-394C-4B15-AA86-7120D6AF9B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B291BDA3-B4DE-4C3D-B971-74A74A02A106}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-2895" windowWidth="29040" windowHeight="15840" xr2:uid="{3126E51C-B0E9-457E-98E2-44FE6544FF4A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" firstSheet="3" activeTab="6" xr2:uid="{3126E51C-B0E9-457E-98E2-44FE6544FF4A}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
@@ -2295,6 +2295,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2302,9 +2305,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3476,18 +3476,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="50" t="s">
         <v>552</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53"/>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
-      <c r="I1" s="53"/>
-      <c r="J1" s="53"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
     </row>
     <row r="2" spans="1:10" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="25" t="s">
@@ -4290,86 +4290,86 @@
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="50" t="s">
+      <c r="A27" s="51" t="s">
         <v>520</v>
       </c>
-      <c r="B27" s="50"/>
-      <c r="C27" s="50"/>
-      <c r="D27" s="50"/>
-      <c r="E27" s="50"/>
-      <c r="F27" s="50"/>
-      <c r="G27" s="50"/>
-      <c r="H27" s="50"/>
-      <c r="I27" s="50"/>
-      <c r="J27" s="50"/>
+      <c r="B27" s="51"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="51"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="51" t="s">
+      <c r="A28" s="52" t="s">
         <v>521</v>
       </c>
-      <c r="B28" s="51"/>
-      <c r="C28" s="51"/>
-      <c r="D28" s="51"/>
-      <c r="E28" s="51"/>
-      <c r="F28" s="51"/>
-      <c r="G28" s="51"/>
-      <c r="H28" s="51"/>
-      <c r="I28" s="51"/>
-      <c r="J28" s="51"/>
+      <c r="B28" s="52"/>
+      <c r="C28" s="52"/>
+      <c r="D28" s="52"/>
+      <c r="E28" s="52"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="52"/>
+      <c r="H28" s="52"/>
+      <c r="I28" s="52"/>
+      <c r="J28" s="52"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="51" t="s">
+      <c r="A29" s="52" t="s">
         <v>522</v>
       </c>
-      <c r="B29" s="51"/>
-      <c r="C29" s="51"/>
-      <c r="D29" s="51"/>
-      <c r="E29" s="51"/>
-      <c r="F29" s="51"/>
-      <c r="G29" s="51"/>
-      <c r="H29" s="51"/>
-      <c r="I29" s="51"/>
-      <c r="J29" s="51"/>
+      <c r="B29" s="52"/>
+      <c r="C29" s="52"/>
+      <c r="D29" s="52"/>
+      <c r="E29" s="52"/>
+      <c r="F29" s="52"/>
+      <c r="G29" s="52"/>
+      <c r="H29" s="52"/>
+      <c r="I29" s="52"/>
+      <c r="J29" s="52"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="51" t="s">
+      <c r="A30" s="52" t="s">
         <v>551</v>
       </c>
-      <c r="B30" s="51"/>
-      <c r="C30" s="51"/>
-      <c r="D30" s="51"/>
-      <c r="E30" s="51"/>
-      <c r="F30" s="51"/>
-      <c r="G30" s="51"/>
-      <c r="H30" s="51"/>
-      <c r="I30" s="51"/>
-      <c r="J30" s="51"/>
+      <c r="B30" s="52"/>
+      <c r="C30" s="52"/>
+      <c r="D30" s="52"/>
+      <c r="E30" s="52"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="52"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="52"/>
+      <c r="J30" s="52"/>
     </row>
     <row r="31" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="52" t="s">
+      <c r="A31" s="53" t="s">
         <v>550</v>
       </c>
-      <c r="B31" s="52"/>
-      <c r="C31" s="52"/>
-      <c r="D31" s="52"/>
-      <c r="E31" s="52"/>
-      <c r="F31" s="52"/>
-      <c r="G31" s="52"/>
-      <c r="H31" s="52"/>
-      <c r="I31" s="52"/>
-      <c r="J31" s="52"/>
+      <c r="B31" s="53"/>
+      <c r="C31" s="53"/>
+      <c r="D31" s="53"/>
+      <c r="E31" s="53"/>
+      <c r="F31" s="53"/>
+      <c r="G31" s="53"/>
+      <c r="H31" s="53"/>
+      <c r="I31" s="53"/>
+      <c r="J31" s="53"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A31:J31"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A27:J27"/>
     <mergeCell ref="A28:J28"/>
     <mergeCell ref="A29:J29"/>
     <mergeCell ref="A30:J30"/>
-    <mergeCell ref="A31:J31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -10571,26 +10571,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d7940701-fd28-48c6-89b6-2769869457dd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE3B5FF1D6D93545B0A9BE76E04A5739" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b213452e5774ccb18cdbac914376359f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af" xmlns:ns3="d7940701-fd28-48c6-89b6-2769869457dd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="94bb0651eba29840b02d7d9879aff2b0" ns2:_="" ns3:_="">
     <xsd:import namespace="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
@@ -10785,32 +10765,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F179CFA0-01D1-49C4-829E-9CD6990EDE07}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="d7940701-fd28-48c6-89b6-2769869457dd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C242F3B7-E13F-47B3-89BF-DC7F2A584373}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d7940701-fd28-48c6-89b6-2769869457dd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14D4D638-0E0C-48CA-BE88-3BE2B56E957A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10827,4 +10802,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C242F3B7-E13F-47B3-89BF-DC7F2A584373}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F179CFA0-01D1-49C4-829E-9CD6990EDE07}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="d7940701-fd28-48c6-89b6-2769869457dd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updating files for resubmission
</commit_message>
<xml_diff>
--- a/data/disruptors_supplementary_data_tables_s1-s5.xlsx
+++ b/data/disruptors_supplementary_data_tables_s1-s5.xlsx
@@ -6543,11 +6543,11 @@
         <v>3300</v>
       </c>
       <c r="K2" s="7">
-        <f>IF(OR(F2="species", F2="genus"), (I2*10^4)/J2,"NA")</f>
+        <f t="shared" ref="K2:K33" si="0">IF(OR(F2="species", F2="genus"), (I2*10^4)/J2,"NA")</f>
         <v>6.0606060606060606</v>
       </c>
       <c r="L2" s="7">
-        <f>IF(H2="percent", I2/(J2/10^6), "NA")</f>
+        <f t="shared" ref="L2:L33" si="1">IF(H2="percent", I2/(J2/10^6), "NA")</f>
         <v>606.06060606060612</v>
       </c>
       <c r="M2" t="s">
@@ -6599,11 +6599,11 @@
         <v>3300</v>
       </c>
       <c r="K3" s="7">
-        <f>IF(OR(F3="species", F3="genus"), (I3*10^4)/J3,"NA")</f>
+        <f t="shared" si="0"/>
         <v>15.151515151515152</v>
       </c>
       <c r="L3" s="7">
-        <f>IF(H3="percent", I3/(J3/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>1515.1515151515152</v>
       </c>
       <c r="M3" t="s">
@@ -6655,11 +6655,11 @@
         <v>3300</v>
       </c>
       <c r="K4" s="7">
-        <f>IF(OR(F4="species", F4="genus"), (I4*10^4)/J4,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-84.848484848484844</v>
       </c>
       <c r="L4" s="7">
-        <f>IF(H4="percent", I4/(J4/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-8484.8484848484841</v>
       </c>
       <c r="M4" t="s">
@@ -6711,11 +6711,11 @@
         <v>3300</v>
       </c>
       <c r="K5" s="7">
-        <f>IF(OR(F5="species", F5="genus"), (I5*10^4)/J5,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-30.303030303030305</v>
       </c>
       <c r="L5" s="7">
-        <f>IF(H5="percent", I5/(J5/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-3030.3030303030305</v>
       </c>
       <c r="M5" t="s">
@@ -6767,11 +6767,11 @@
         <v>3300</v>
       </c>
       <c r="K6" s="7">
-        <f>IF(OR(F6="species", F6="genus"), (I6*10^4)/J6,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-15.151515151515152</v>
       </c>
       <c r="L6" s="7">
-        <f>IF(H6="percent", I6/(J6/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-1515.1515151515152</v>
       </c>
       <c r="M6" t="s">
@@ -6823,11 +6823,11 @@
         <v>300</v>
       </c>
       <c r="K7" s="7">
-        <f>IF(OR(F7="species", F7="genus"), (I7*10^4)/J7,"NA")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L7" s="7">
-        <f>IF(H7="percent", I7/(J7/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M7" t="s">
@@ -6879,11 +6879,11 @@
         <v>300</v>
       </c>
       <c r="K8" s="7">
-        <f>IF(OR(F8="species", F8="genus"), (I8*10^4)/J8,"NA")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L8" s="7">
-        <f>IF(H8="percent", I8/(J8/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M8" t="s">
@@ -6929,11 +6929,11 @@
         <v>300</v>
       </c>
       <c r="K9" s="7">
-        <f>IF(OR(F9="species", F9="genus"), (I9*10^4)/J9,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-1066.6666666666667</v>
       </c>
       <c r="L9" s="7">
-        <f>IF(H9="percent", I9/(J9/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-106666.66666666667</v>
       </c>
       <c r="O9" t="s">
@@ -6976,11 +6976,11 @@
         <v>300</v>
       </c>
       <c r="K10" s="7">
-        <f>IF(OR(F10="species", F10="genus"), (I10*10^4)/J10,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-900</v>
       </c>
       <c r="L10" s="7">
-        <f>IF(H10="percent", I10/(J10/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-90000.000000000015</v>
       </c>
       <c r="M10" t="s">
@@ -7026,11 +7026,11 @@
         <v>300</v>
       </c>
       <c r="K11" s="7">
-        <f>IF(OR(F11="species", F11="genus"), (I11*10^4)/J11,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-586.66666666666663</v>
       </c>
       <c r="L11" s="7">
-        <f>IF(H11="percent", I11/(J11/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-58666.666666666679</v>
       </c>
       <c r="M11" t="s">
@@ -7076,11 +7076,11 @@
         <v>300</v>
       </c>
       <c r="K12" s="7">
-        <f>IF(OR(F12="species", F12="genus"), (I12*10^4)/J12,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-466.66666666666669</v>
       </c>
       <c r="L12" s="7">
-        <f>IF(H12="percent", I12/(J12/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-46666.666666666672</v>
       </c>
       <c r="O12" t="s">
@@ -7123,11 +7123,11 @@
         <v>300</v>
       </c>
       <c r="K13" s="7">
-        <f>IF(OR(F13="species", F13="genus"), (I13*10^4)/J13,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-433.33333333333331</v>
       </c>
       <c r="L13" s="7">
-        <f>IF(H13="percent", I13/(J13/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-43333.333333333336</v>
       </c>
       <c r="M13" t="s">
@@ -7173,11 +7173,11 @@
         <v>300</v>
       </c>
       <c r="K14" s="7">
-        <f>IF(OR(F14="species", F14="genus"), (I14*10^4)/J14,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-260</v>
       </c>
       <c r="L14" s="7">
-        <f>IF(H14="percent", I14/(J14/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-26000</v>
       </c>
       <c r="M14" t="s">
@@ -7223,11 +7223,11 @@
         <v>300</v>
       </c>
       <c r="K15" s="7">
-        <f>IF(OR(F15="species", F15="genus"), (I15*10^4)/J15,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-126.66666666666667</v>
       </c>
       <c r="L15" s="7">
-        <f>IF(H15="percent", I15/(J15/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-12666.666666666668</v>
       </c>
       <c r="M15" t="s">
@@ -7273,11 +7273,11 @@
         <v>200</v>
       </c>
       <c r="K16" s="7" t="str">
-        <f>IF(OR(F16="species", F16="genus"), (I16*10^4)/J16,"NA")</f>
+        <f t="shared" si="0"/>
         <v>NA</v>
       </c>
       <c r="L16" s="7">
-        <f>IF(H16="percent", I16/(J16/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-415000</v>
       </c>
       <c r="M16" t="s">
@@ -7323,11 +7323,11 @@
         <v>200</v>
       </c>
       <c r="K17" s="7">
-        <f>IF(OR(F17="species", F17="genus"), (I17*10^4)/J17,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-2500</v>
       </c>
       <c r="L17" s="7">
-        <f>IF(H17="percent", I17/(J17/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-250000</v>
       </c>
       <c r="O17" t="s">
@@ -7370,11 +7370,11 @@
         <v>200</v>
       </c>
       <c r="K18" s="7" t="str">
-        <f>IF(OR(F18="species", F18="genus"), (I18*10^4)/J18,"NA")</f>
+        <f t="shared" si="0"/>
         <v>NA</v>
       </c>
       <c r="L18" s="7">
-        <f>IF(H18="percent", I18/(J18/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-150000</v>
       </c>
       <c r="M18" t="s">
@@ -7420,11 +7420,11 @@
         <v>200</v>
       </c>
       <c r="K19" s="7">
-        <f>IF(OR(F19="species", F19="genus"), (I19*10^4)/J19,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-80.500000000000014</v>
       </c>
       <c r="L19" s="7">
-        <f>IF(H19="percent", I19/(J19/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-8050</v>
       </c>
       <c r="M19" t="s">
@@ -7470,11 +7470,11 @@
         <v>200</v>
       </c>
       <c r="K20" s="7">
-        <f>IF(OR(F20="species", F20="genus"), (I20*10^4)/J20,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-77</v>
       </c>
       <c r="L20" s="7">
-        <f>IF(H20="percent", I20/(J20/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-7700</v>
       </c>
       <c r="M20" t="s">
@@ -7520,11 +7520,11 @@
         <v>200</v>
       </c>
       <c r="K21" s="7">
-        <f>IF(OR(F21="species", F21="genus"), (I21*10^4)/J21,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-44</v>
       </c>
       <c r="L21" s="7">
-        <f>IF(H21="percent", I21/(J21/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-4400</v>
       </c>
       <c r="M21" t="s">
@@ -7570,11 +7570,11 @@
         <v>200</v>
       </c>
       <c r="K22" s="7">
-        <f>IF(OR(F22="species", F22="genus"), (I22*10^4)/J22,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-29</v>
       </c>
       <c r="L22" s="7">
-        <f>IF(H22="percent", I22/(J22/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-2899.9999999999995</v>
       </c>
       <c r="M22" t="s">
@@ -7620,11 +7620,11 @@
         <v>200</v>
       </c>
       <c r="K23" s="7">
-        <f>IF(OR(F23="species", F23="genus"), (I23*10^4)/J23,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-25</v>
       </c>
       <c r="L23" s="7">
-        <f>IF(H23="percent", I23/(J23/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-2500</v>
       </c>
       <c r="O23" t="s">
@@ -7667,11 +7667,11 @@
         <v>200</v>
       </c>
       <c r="K24" s="7">
-        <f>IF(OR(F24="species", F24="genus"), (I24*10^4)/J24,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-22.5</v>
       </c>
       <c r="L24" s="7">
-        <f>IF(H24="percent", I24/(J24/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-2250</v>
       </c>
       <c r="M24" t="s">
@@ -7714,11 +7714,11 @@
         <v>200</v>
       </c>
       <c r="K25" s="7">
-        <f>IF(OR(F25="species", F25="genus"), (I25*10^4)/J25,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-8.5000000000000018</v>
       </c>
       <c r="L25" s="7">
-        <f>IF(H25="percent", I25/(J25/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-850</v>
       </c>
       <c r="M25" t="s">
@@ -7761,11 +7761,11 @@
         <v>200</v>
       </c>
       <c r="K26" s="7">
-        <f>IF(OR(F26="species", F26="genus"), (I26*10^4)/J26,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-0.5</v>
       </c>
       <c r="L26" s="7">
-        <f>IF(H26="percent", I26/(J26/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-50</v>
       </c>
     </row>
@@ -7805,11 +7805,11 @@
         <v>200</v>
       </c>
       <c r="K27" s="7">
-        <f>IF(OR(F27="species", F27="genus"), (I27*10^4)/J27,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-50</v>
       </c>
       <c r="L27" s="7">
-        <f>IF(H27="percent", I27/(J27/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-5000</v>
       </c>
       <c r="M27" t="s">
@@ -7852,11 +7852,11 @@
         <v>500000</v>
       </c>
       <c r="K28" s="7">
-        <f>IF(OR(F28="species", F28="genus"), (I28*10^4)/J28,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-0.01</v>
       </c>
       <c r="L28" s="7">
-        <f>IF(H28="percent", I28/(J28/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="M28" t="s">
@@ -7899,11 +7899,11 @@
         <v>500000</v>
       </c>
       <c r="K29" s="7">
-        <f>IF(OR(F29="species", F29="genus"), (I29*10^4)/J29,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-0.22</v>
       </c>
       <c r="L29" s="7">
-        <f>IF(H29="percent", I29/(J29/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-22</v>
       </c>
       <c r="M29" t="s">
@@ -7946,11 +7946,11 @@
         <v>500000</v>
       </c>
       <c r="K30" s="7">
-        <f>IF(OR(F30="species", F30="genus"), (I30*10^4)/J30,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-0.72</v>
       </c>
       <c r="L30" s="7">
-        <f>IF(H30="percent", I30/(J30/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-72</v>
       </c>
       <c r="M30" t="s">
@@ -7993,11 +7993,11 @@
         <v>500000</v>
       </c>
       <c r="K31" s="7">
-        <f>IF(OR(F31="species", F31="genus"), (I31*10^4)/J31,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-0.98</v>
       </c>
       <c r="L31" s="7">
-        <f>IF(H31="percent", I31/(J31/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-98</v>
       </c>
       <c r="M31" t="s">
@@ -8040,11 +8040,11 @@
         <v>500000</v>
       </c>
       <c r="K32" s="7">
-        <f>IF(OR(F32="species", F32="genus"), (I32*10^4)/J32,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-0.84</v>
       </c>
       <c r="L32" s="7">
-        <f>IF(H32="percent", I32/(J32/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-84</v>
       </c>
       <c r="M32" t="s">
@@ -8087,11 +8087,11 @@
         <v>100000</v>
       </c>
       <c r="K33" s="7">
-        <f>IF(OR(F33="species", F33="genus"), (I33*10^4)/J33,"NA")</f>
+        <f t="shared" si="0"/>
         <v>-7.7</v>
       </c>
       <c r="L33" s="7">
-        <f>IF(H33="percent", I33/(J33/10^6), "NA")</f>
+        <f t="shared" si="1"/>
         <v>-770</v>
       </c>
     </row>
@@ -8131,11 +8131,11 @@
         <v>100000</v>
       </c>
       <c r="K34" s="7">
-        <f>IF(OR(F34="species", F34="genus"), (I34*10^4)/J34,"NA")</f>
+        <f t="shared" ref="K34:K65" si="2">IF(OR(F34="species", F34="genus"), (I34*10^4)/J34,"NA")</f>
         <v>-1.6</v>
       </c>
       <c r="L34" s="7">
-        <f>IF(H34="percent", I34/(J34/10^6), "NA")</f>
+        <f t="shared" ref="L34:L65" si="3">IF(H34="percent", I34/(J34/10^6), "NA")</f>
         <v>-160</v>
       </c>
     </row>
@@ -8175,11 +8175,11 @@
         <v>100000</v>
       </c>
       <c r="K35" s="7">
-        <f>IF(OR(F35="species", F35="genus"), (I35*10^4)/J35,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-1.5</v>
       </c>
       <c r="L35" s="7">
-        <f>IF(H35="percent", I35/(J35/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-150</v>
       </c>
     </row>
@@ -8219,11 +8219,11 @@
         <v>150000</v>
       </c>
       <c r="K36" s="7">
-        <f>IF(OR(F36="species", F36="genus"), (I36*10^4)/J36,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-4.333333333333333</v>
       </c>
       <c r="L36" s="7">
-        <f>IF(H36="percent", I36/(J36/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-433.33333333333337</v>
       </c>
     </row>
@@ -8263,11 +8263,11 @@
         <v>150000</v>
       </c>
       <c r="K37" s="7">
-        <f>IF(OR(F37="species", F37="genus"), (I37*10^4)/J37,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-2.2000000000000002</v>
       </c>
       <c r="L37" s="7">
-        <f>IF(H37="percent", I37/(J37/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-220</v>
       </c>
     </row>
@@ -8307,11 +8307,11 @@
         <v>150000</v>
       </c>
       <c r="K38" s="7">
-        <f>IF(OR(F38="species", F38="genus"), (I38*10^4)/J38,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-1.3333333333333333</v>
       </c>
       <c r="L38" s="7">
-        <f>IF(H38="percent", I38/(J38/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-133.33333333333334</v>
       </c>
     </row>
@@ -8351,11 +8351,11 @@
         <v>150000</v>
       </c>
       <c r="K39" s="7">
-        <f>IF(OR(F39="species", F39="genus"), (I39*10^4)/J39,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-6.6666666666666666E-2</v>
       </c>
       <c r="L39" s="7">
-        <f>IF(H39="percent", I39/(J39/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-6.666666666666667</v>
       </c>
     </row>
@@ -8395,11 +8395,11 @@
         <v>30</v>
       </c>
       <c r="K40" s="7">
-        <f>IF(OR(F40="species", F40="genus"), (I40*10^4)/J40,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-13333.333333333334</v>
       </c>
       <c r="L40" s="7">
-        <f>IF(H40="percent", I40/(J40/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-1333333.3333333333</v>
       </c>
     </row>
@@ -8439,11 +8439,11 @@
         <v>30</v>
       </c>
       <c r="K41" s="7">
-        <f>IF(OR(F41="species", F41="genus"), (I41*10^4)/J41,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-13333.333333333334</v>
       </c>
       <c r="L41" s="7">
-        <f>IF(H41="percent", I41/(J41/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-1333333.3333333333</v>
       </c>
     </row>
@@ -8483,11 +8483,11 @@
         <v>30</v>
       </c>
       <c r="K42" s="7">
-        <f>IF(OR(F42="species", F42="genus"), (I42*10^4)/J42,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-13000</v>
       </c>
       <c r="L42" s="7">
-        <f>IF(H42="percent", I42/(J42/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-1300000</v>
       </c>
     </row>
@@ -8527,11 +8527,11 @@
         <v>30</v>
       </c>
       <c r="K43" s="7">
-        <f>IF(OR(F43="species", F43="genus"), (I43*10^4)/J43,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-25000</v>
       </c>
       <c r="L43" s="7">
-        <f>IF(H43="percent", I43/(J43/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-2500000</v>
       </c>
       <c r="M43" t="s">
@@ -8574,11 +8574,11 @@
         <v>500000</v>
       </c>
       <c r="K44" s="7">
-        <f>IF(OR(F44="species", F44="genus"), (I44*10^4)/J44,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.4</v>
       </c>
       <c r="L44" s="7">
-        <f>IF(H44="percent", I44/(J44/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-40</v>
       </c>
     </row>
@@ -8618,11 +8618,11 @@
         <v>500000</v>
       </c>
       <c r="K45" s="7">
-        <f>IF(OR(F45="species", F45="genus"), (I45*10^4)/J45,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.44</v>
       </c>
       <c r="L45" s="7">
-        <f>IF(H45="percent", I45/(J45/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-44</v>
       </c>
     </row>
@@ -8662,11 +8662,11 @@
         <v>75000000</v>
       </c>
       <c r="K46" s="7">
-        <f>IF(OR(F46="species", F46="genus"), (I46*10^4)/J46,"NA")</f>
+        <f t="shared" si="2"/>
         <v>0.02</v>
       </c>
       <c r="L46" s="7">
-        <f>IF(H46="percent", I46/(J46/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>2</v>
       </c>
       <c r="M46" t="s">
@@ -8709,11 +8709,11 @@
         <v>75000000</v>
       </c>
       <c r="K47" s="7" t="str">
-        <f>IF(OR(F47="species", F47="genus"), (I47*10^4)/J47,"NA")</f>
+        <f t="shared" si="2"/>
         <v>NA</v>
       </c>
       <c r="L47" s="7">
-        <f>IF(H47="percent", I47/(J47/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>2.1466666666666665</v>
       </c>
       <c r="M47" t="s">
@@ -8756,11 +8756,11 @@
         <v>1000000</v>
       </c>
       <c r="K48" s="7">
-        <f>IF(OR(F48="species", F48="genus"), (I48*10^4)/J48,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.2</v>
       </c>
       <c r="L48" s="7">
-        <f>IF(H48="percent", I48/(J48/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-20</v>
       </c>
     </row>
@@ -8800,11 +8800,11 @@
         <v>500000</v>
       </c>
       <c r="K49" s="7">
-        <f>IF(OR(F49="species", F49="genus"), (I49*10^4)/J49,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.5</v>
       </c>
       <c r="L49" s="7">
-        <f>IF(H49="percent", I49/(J49/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-50</v>
       </c>
     </row>
@@ -8844,11 +8844,11 @@
         <v>500000</v>
       </c>
       <c r="K50" s="7">
-        <f>IF(OR(F50="species", F50="genus"), (I50*10^4)/J50,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.44</v>
       </c>
       <c r="L50" s="7">
-        <f>IF(H50="percent", I50/(J50/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-44</v>
       </c>
     </row>
@@ -8888,11 +8888,11 @@
         <v>500000</v>
       </c>
       <c r="K51" s="7">
-        <f>IF(OR(F51="species", F51="genus"), (I51*10^4)/J51,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.4</v>
       </c>
       <c r="L51" s="7">
-        <f>IF(H51="percent", I51/(J51/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-40</v>
       </c>
     </row>
@@ -8932,11 +8932,11 @@
         <v>500000</v>
       </c>
       <c r="K52" s="7">
-        <f>IF(OR(F52="species", F52="genus"), (I52*10^4)/J52,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.3</v>
       </c>
       <c r="L52" s="7">
-        <f>IF(H52="percent", I52/(J52/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-30</v>
       </c>
     </row>
@@ -8975,11 +8975,11 @@
         <v>500000</v>
       </c>
       <c r="K53" s="7">
-        <f>IF(OR(F53="species", F53="genus"), (I53*10^4)/J53,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.52</v>
       </c>
       <c r="L53" s="7">
-        <f>IF(H53="percent", I53/(J53/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-52</v>
       </c>
     </row>
@@ -9019,11 +9019,11 @@
         <v>85000</v>
       </c>
       <c r="K54" s="7">
-        <f>IF(OR(F54="species", F54="genus"), (I54*10^4)/J54,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-9.4117647058823533</v>
       </c>
       <c r="L54" s="7">
-        <f>IF(H54="percent", I54/(J54/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-941.17647058823525</v>
       </c>
     </row>
@@ -9063,11 +9063,11 @@
         <v>85000</v>
       </c>
       <c r="K55" s="7">
-        <f>IF(OR(F55="species", F55="genus"), (I55*10^4)/J55,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-8.5882352941176467</v>
       </c>
       <c r="L55" s="7">
-        <f>IF(H55="percent", I55/(J55/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-858.82352941176464</v>
       </c>
     </row>
@@ -9107,11 +9107,11 @@
         <v>85000</v>
       </c>
       <c r="K56" s="7">
-        <f>IF(OR(F56="species", F56="genus"), (I56*10^4)/J56,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-5.5294117647058822</v>
       </c>
       <c r="L56" s="7">
-        <f>IF(H56="percent", I56/(J56/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-552.94117647058818</v>
       </c>
     </row>
@@ -9151,11 +9151,11 @@
         <v>1090000</v>
       </c>
       <c r="K57" s="7">
-        <f>IF(OR(F57="species", F57="genus"), (I57*10^4)/J57,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.56880733944954132</v>
       </c>
       <c r="L57" s="7">
-        <f>IF(H57="percent", I57/(J57/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-56.880733944954123</v>
       </c>
       <c r="M57" t="s">
@@ -9198,11 +9198,11 @@
         <v>1090000</v>
       </c>
       <c r="K58" s="7">
-        <f>IF(OR(F58="species", F58="genus"), (I58*10^4)/J58,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.46788990825688076</v>
       </c>
       <c r="L58" s="7">
-        <f>IF(H58="percent", I58/(J58/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-46.788990825688067</v>
       </c>
       <c r="M58" t="s">
@@ -9245,11 +9245,11 @@
         <v>1090000</v>
       </c>
       <c r="K59" s="7">
-        <f>IF(OR(F59="species", F59="genus"), (I59*10^4)/J59,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.30275229357798167</v>
       </c>
       <c r="L59" s="7">
-        <f>IF(H59="percent", I59/(J59/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-30.275229357798164</v>
       </c>
       <c r="M59" t="s">
@@ -9292,11 +9292,11 @@
         <v>60000</v>
       </c>
       <c r="K60" s="7">
-        <f>IF(OR(F60="species", F60="genus"), (I60*10^4)/J60,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-15.833333333333334</v>
       </c>
       <c r="L60" s="7">
-        <f>IF(H60="percent", I60/(J60/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-1583.3333333333335</v>
       </c>
     </row>
@@ -9336,11 +9336,11 @@
         <v>60000</v>
       </c>
       <c r="K61" s="7">
-        <f>IF(OR(F61="species", F61="genus"), (I61*10^4)/J61,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-13.833333333333334</v>
       </c>
       <c r="L61" s="7">
-        <f>IF(H61="percent", I61/(J61/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-1383.3333333333335</v>
       </c>
     </row>
@@ -9380,11 +9380,11 @@
         <v>60000</v>
       </c>
       <c r="K62" s="7" t="str">
-        <f>IF(OR(F62="species", F62="genus"), (I62*10^4)/J62,"NA")</f>
+        <f t="shared" si="2"/>
         <v>NA</v>
       </c>
       <c r="L62" s="7">
-        <f>IF(H62="percent", I62/(J62/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-1166.6666666666667</v>
       </c>
     </row>
@@ -9424,11 +9424,11 @@
         <v>60000</v>
       </c>
       <c r="K63" s="7">
-        <f>IF(OR(F63="species", F63="genus"), (I63*10^4)/J63,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-10.333333333333334</v>
       </c>
       <c r="L63" s="7">
-        <f>IF(H63="percent", I63/(J63/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-1033.3333333333335</v>
       </c>
     </row>
@@ -9468,11 +9468,11 @@
         <v>60000</v>
       </c>
       <c r="K64" s="7">
-        <f>IF(OR(F64="species", F64="genus"), (I64*10^4)/J64,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-9.3333333333333339</v>
       </c>
       <c r="L64" s="7">
-        <f>IF(H64="percent", I64/(J64/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-933.33333333333337</v>
       </c>
     </row>
@@ -9512,11 +9512,11 @@
         <v>1500000</v>
       </c>
       <c r="K65" s="7">
-        <f>IF(OR(F65="species", F65="genus"), (I65*10^4)/J65,"NA")</f>
+        <f t="shared" si="2"/>
         <v>-0.32</v>
       </c>
       <c r="L65" s="7">
-        <f>IF(H65="percent", I65/(J65/10^6), "NA")</f>
+        <f t="shared" si="3"/>
         <v>-32</v>
       </c>
     </row>
@@ -9556,11 +9556,11 @@
         <v>1500000</v>
       </c>
       <c r="K66" s="7">
-        <f>IF(OR(F66="species", F66="genus"), (I66*10^4)/J66,"NA")</f>
+        <f t="shared" ref="K66:K97" si="4">IF(OR(F66="species", F66="genus"), (I66*10^4)/J66,"NA")</f>
         <v>-0.22666666666666666</v>
       </c>
       <c r="L66" s="7">
-        <f>IF(H66="percent", I66/(J66/10^6), "NA")</f>
+        <f t="shared" ref="L66:L97" si="5">IF(H66="percent", I66/(J66/10^6), "NA")</f>
         <v>-22.666666666666668</v>
       </c>
     </row>
@@ -9600,11 +9600,11 @@
         <v>1500000</v>
       </c>
       <c r="K67" s="7">
-        <f>IF(OR(F67="species", F67="genus"), (I67*10^4)/J67,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.16666666666666666</v>
       </c>
       <c r="L67" s="7">
-        <f>IF(H67="percent", I67/(J67/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-16.666666666666668</v>
       </c>
     </row>
@@ -9644,11 +9644,11 @@
         <v>4000000</v>
       </c>
       <c r="K68" s="7">
-        <f>IF(OR(F68="species", F68="genus"), (I68*10^4)/J68,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-9.7500000000000003E-2</v>
       </c>
       <c r="L68" s="7">
-        <f>IF(H68="percent", I68/(J68/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-9.75</v>
       </c>
     </row>
@@ -9688,11 +9688,11 @@
         <v>4000000</v>
       </c>
       <c r="K69" s="7">
-        <f>IF(OR(F69="species", F69="genus"), (I69*10^4)/J69,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-7.7499999999999999E-2</v>
       </c>
       <c r="L69" s="7">
-        <f>IF(H69="percent", I69/(J69/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-7.75</v>
       </c>
       <c r="Z69" s="8"/>
@@ -9733,11 +9733,11 @@
         <v>4000000</v>
       </c>
       <c r="K70" s="7">
-        <f>IF(OR(F70="species", F70="genus"), (I70*10^4)/J70,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-3.5000000000000003E-2</v>
       </c>
       <c r="L70" s="7">
-        <f>IF(H70="percent", I70/(J70/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-3.5</v>
       </c>
       <c r="Z70" s="8"/>
@@ -9778,11 +9778,11 @@
         <v>100000</v>
       </c>
       <c r="K71" s="7">
-        <f>IF(OR(F71="species", F71="genus"), (I71*10^4)/J71,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
       <c r="L71" s="7">
-        <f>IF(H71="percent", I71/(J71/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-500</v>
       </c>
       <c r="Z71" s="8"/>
@@ -9823,11 +9823,11 @@
         <v>100000</v>
       </c>
       <c r="K72" s="7">
-        <f>IF(OR(F72="species", F72="genus"), (I72*10^4)/J72,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-3.1</v>
       </c>
       <c r="L72" s="7">
-        <f>IF(H72="percent", I72/(J72/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-310</v>
       </c>
       <c r="Y72" s="8"/>
@@ -9869,11 +9869,11 @@
         <v>100000</v>
       </c>
       <c r="K73" s="7">
-        <f>IF(OR(F73="species", F73="genus"), (I73*10^4)/J73,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-4</v>
       </c>
       <c r="L73" s="7">
-        <f>IF(H73="percent", I73/(J73/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-400</v>
       </c>
       <c r="Z73" s="8"/>
@@ -9914,11 +9914,11 @@
         <v>100000</v>
       </c>
       <c r="K74" s="7">
-        <f>IF(OR(F74="species", F74="genus"), (I74*10^4)/J74,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-3.5</v>
       </c>
       <c r="L74" s="7">
-        <f>IF(H74="percent", I74/(J74/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-350</v>
       </c>
       <c r="Y74" s="8"/>
@@ -9960,11 +9960,11 @@
         <v>100000</v>
       </c>
       <c r="K75" s="7">
-        <f>IF(OR(F75="species", F75="genus"), (I75*10^4)/J75,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-1.8</v>
       </c>
       <c r="L75" s="7">
-        <f>IF(H75="percent", I75/(J75/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-180</v>
       </c>
     </row>
@@ -10004,11 +10004,11 @@
         <v>1500000</v>
       </c>
       <c r="K76" s="7">
-        <f>IF(OR(F76="species", F76="genus"), (I76*10^4)/J76,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.24</v>
       </c>
       <c r="L76" s="7">
-        <f>IF(H76="percent", I76/(J76/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-24</v>
       </c>
     </row>
@@ -10048,11 +10048,11 @@
         <v>1500000</v>
       </c>
       <c r="K77" s="7">
-        <f>IF(OR(F77="species", F77="genus"), (I77*10^4)/J77,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.19333333333333333</v>
       </c>
       <c r="L77" s="7">
-        <f>IF(H77="percent", I77/(J77/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-19.333333333333332</v>
       </c>
     </row>
@@ -10092,11 +10092,11 @@
         <v>100000</v>
       </c>
       <c r="K78" s="7">
-        <f>IF(OR(F78="species", F78="genus"), (I78*10^4)/J78,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-3.2</v>
       </c>
       <c r="L78" s="7">
-        <f>IF(H78="percent", I78/(J78/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-320</v>
       </c>
     </row>
@@ -10136,11 +10136,11 @@
         <v>500000</v>
       </c>
       <c r="K79" s="7">
-        <f>IF(OR(F79="species", F79="genus"), (I79*10^4)/J79,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.42</v>
       </c>
       <c r="L79" s="7">
-        <f>IF(H79="percent", I79/(J79/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-42</v>
       </c>
     </row>
@@ -10180,11 +10180,11 @@
         <v>500000</v>
       </c>
       <c r="K80" s="7">
-        <f>IF(OR(F80="species", F80="genus"), (I80*10^4)/J80,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.18</v>
       </c>
       <c r="L80" s="7">
-        <f>IF(H80="percent", I80/(J80/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-18</v>
       </c>
     </row>
@@ -10224,11 +10224,11 @@
         <v>1000000</v>
       </c>
       <c r="K81" s="7">
-        <f>IF(OR(F81="species", F81="genus"), (I81*10^4)/J81,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.25</v>
       </c>
       <c r="L81" s="7">
-        <f>IF(H81="percent", I81/(J81/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-25</v>
       </c>
     </row>
@@ -10268,11 +10268,11 @@
         <v>1000000</v>
       </c>
       <c r="K82" s="7">
-        <f>IF(OR(F82="species", F82="genus"), (I82*10^4)/J82,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.22</v>
       </c>
       <c r="L82" s="7">
-        <f>IF(H82="percent", I82/(J82/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-22</v>
       </c>
     </row>
@@ -10311,11 +10311,11 @@
         <v>500000</v>
       </c>
       <c r="K83" s="7">
-        <f>IF(OR(F83="species", F83="genus"), (I83*10^4)/J83,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-1.7</v>
       </c>
       <c r="L83" s="7">
-        <f>IF(H83="percent", I83/(J83/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-170</v>
       </c>
     </row>
@@ -10354,11 +10354,11 @@
         <v>500000</v>
       </c>
       <c r="K84" s="7">
-        <f>IF(OR(F84="species", F84="genus"), (I84*10^4)/J84,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.98</v>
       </c>
       <c r="L84" s="7">
-        <f>IF(H84="percent", I84/(J84/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-98</v>
       </c>
     </row>
@@ -10398,11 +10398,11 @@
         <v>500000</v>
       </c>
       <c r="K85" s="7">
-        <f>IF(OR(F85="species", F85="genus"), (I85*10^4)/J85,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-1.1399999999999999</v>
       </c>
       <c r="L85" s="7">
-        <f>IF(H85="percent", I85/(J85/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-114</v>
       </c>
     </row>
@@ -10442,11 +10442,11 @@
         <v>500000</v>
       </c>
       <c r="K86" s="7">
-        <f>IF(OR(F86="species", F86="genus"), (I86*10^4)/J86,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-1.04</v>
       </c>
       <c r="L86" s="7">
-        <f>IF(H86="percent", I86/(J86/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-104</v>
       </c>
     </row>
@@ -10486,11 +10486,11 @@
         <v>500000</v>
       </c>
       <c r="K87" s="7">
-        <f>IF(OR(F87="species", F87="genus"), (I87*10^4)/J87,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.92</v>
       </c>
       <c r="L87" s="7">
-        <f>IF(H87="percent", I87/(J87/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-92</v>
       </c>
     </row>
@@ -10530,11 +10530,11 @@
         <v>60000000</v>
       </c>
       <c r="K88" s="7" t="str">
-        <f>IF(OR(F88="species", F88="genus"), (I88*10^4)/J88,"NA")</f>
+        <f t="shared" si="4"/>
         <v>NA</v>
       </c>
       <c r="L88" s="7">
-        <f>IF(H88="percent", I88/(J88/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>0.58333333333333337</v>
       </c>
       <c r="M88" t="s">
@@ -10577,11 +10577,11 @@
         <v>60000000</v>
       </c>
       <c r="K89" s="7" t="str">
-        <f>IF(OR(F89="species", F89="genus"), (I89*10^4)/J89,"NA")</f>
+        <f t="shared" si="4"/>
         <v>NA</v>
       </c>
       <c r="L89" s="7">
-        <f>IF(H89="percent", I89/(J89/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>1.3333333333333333</v>
       </c>
       <c r="M89" t="s">
@@ -10624,11 +10624,11 @@
         <v>60000000</v>
       </c>
       <c r="K90" s="7" t="str">
-        <f>IF(OR(F90="species", F90="genus"), (I90*10^4)/J90,"NA")</f>
+        <f t="shared" si="4"/>
         <v>NA</v>
       </c>
       <c r="L90" s="7">
-        <f>IF(H90="percent", I90/(J90/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>2.4500000000000002</v>
       </c>
       <c r="M90" t="s">
@@ -10671,11 +10671,11 @@
         <v>60000000</v>
       </c>
       <c r="K91" s="7" t="str">
-        <f>IF(OR(F91="species", F91="genus"), (I91*10^4)/J91,"NA")</f>
+        <f t="shared" si="4"/>
         <v>NA</v>
       </c>
       <c r="L91" s="7">
-        <f>IF(H91="percent", I91/(J91/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>15</v>
       </c>
       <c r="M91" t="s">
@@ -10718,11 +10718,11 @@
         <v>60000000</v>
       </c>
       <c r="K92" s="7">
-        <f>IF(OR(F92="species", F92="genus"), (I92*10^4)/J92,"NA")</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="L92" s="7">
-        <f>IF(H92="percent", I92/(J92/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>200</v>
       </c>
       <c r="M92" t="s">
@@ -10765,11 +10765,11 @@
         <v>60000000</v>
       </c>
       <c r="K93" s="7">
-        <f>IF(OR(F93="species", F93="genus"), (I93*10^4)/J93,"NA")</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="L93" s="7">
-        <f>IF(H93="percent", I93/(J93/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>300</v>
       </c>
       <c r="M93" t="s">
@@ -10811,11 +10811,11 @@
         <v>30000000</v>
       </c>
       <c r="K94" s="7">
-        <f>IF(OR(F94="species", F94="genus"), (I94*10^4)/J94,"NA")</f>
+        <f t="shared" si="4"/>
         <v>0.26666666666666666</v>
       </c>
       <c r="L94" s="7">
-        <f>IF(H94="percent", I94/(J94/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>26.666666666666668</v>
       </c>
       <c r="M94" t="s">
@@ -10858,11 +10858,11 @@
         <v>2600000</v>
       </c>
       <c r="K95" s="7">
-        <f>IF(OR(F95="species", F95="genus"), (I95*10^4)/J95,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.25</v>
       </c>
       <c r="L95" s="7">
-        <f>IF(H95="percent", I95/(J95/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-25</v>
       </c>
     </row>
@@ -10902,11 +10902,11 @@
         <v>2600000</v>
       </c>
       <c r="K96" s="7">
-        <f>IF(OR(F96="species", F96="genus"), (I96*10^4)/J96,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.23076923076923078</v>
       </c>
       <c r="L96" s="7">
-        <f>IF(H96="percent", I96/(J96/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-23.076923076923077</v>
       </c>
       <c r="M96" t="s">
@@ -10949,11 +10949,11 @@
         <v>2600000</v>
       </c>
       <c r="K97" s="7">
-        <f>IF(OR(F97="species", F97="genus"), (I97*10^4)/J97,"NA")</f>
+        <f t="shared" si="4"/>
         <v>-0.22692307692307692</v>
       </c>
       <c r="L97" s="7">
-        <f>IF(H97="percent", I97/(J97/10^6), "NA")</f>
+        <f t="shared" si="5"/>
         <v>-22.69230769230769</v>
       </c>
     </row>
@@ -10993,11 +10993,11 @@
         <v>2600000</v>
       </c>
       <c r="K98" s="7">
-        <f>IF(OR(F98="species", F98="genus"), (I98*10^4)/J98,"NA")</f>
+        <f t="shared" ref="K98:K129" si="6">IF(OR(F98="species", F98="genus"), (I98*10^4)/J98,"NA")</f>
         <v>-0.22307692307692309</v>
       </c>
       <c r="L98" s="7">
-        <f>IF(H98="percent", I98/(J98/10^6), "NA")</f>
+        <f t="shared" ref="L98:L107" si="7">IF(H98="percent", I98/(J98/10^6), "NA")</f>
         <v>-22.307692307692307</v>
       </c>
     </row>
@@ -11037,11 +11037,11 @@
         <v>500000</v>
       </c>
       <c r="K99" s="7">
-        <f>IF(OR(F99="species", F99="genus"), (I99*10^4)/J99,"NA")</f>
+        <f t="shared" si="6"/>
         <v>-1</v>
       </c>
       <c r="L99" s="7">
-        <f>IF(H99="percent", I99/(J99/10^6), "NA")</f>
+        <f t="shared" si="7"/>
         <v>-100</v>
       </c>
       <c r="M99" t="s">
@@ -11084,11 +11084,11 @@
         <v>1000000</v>
       </c>
       <c r="K100" s="7">
-        <f>IF(OR(F100="species", F100="genus"), (I100*10^4)/J100,"NA")</f>
+        <f t="shared" si="6"/>
         <v>-0.5</v>
       </c>
       <c r="L100" s="7">
-        <f>IF(H100="percent", I100/(J100/10^6), "NA")</f>
+        <f t="shared" si="7"/>
         <v>-50</v>
       </c>
       <c r="M100" t="s">
@@ -11131,11 +11131,11 @@
         <v>1000000</v>
       </c>
       <c r="K101" s="7">
-        <f>IF(OR(F101="species", F101="genus"), (I101*10^4)/J101,"NA")</f>
+        <f t="shared" si="6"/>
         <v>-0.49</v>
       </c>
       <c r="L101" s="7">
-        <f>IF(H101="percent", I101/(J101/10^6), "NA")</f>
+        <f t="shared" si="7"/>
         <v>-49</v>
       </c>
     </row>
@@ -11175,11 +11175,11 @@
         <v>40000000</v>
       </c>
       <c r="K102" s="7" t="str">
-        <f>IF(OR(F102="species", F102="genus"), (I102*10^4)/J102,"NA")</f>
+        <f t="shared" si="6"/>
         <v>NA</v>
       </c>
       <c r="L102" s="7">
-        <f>IF(H102="percent", I102/(J102/10^6), "NA")</f>
+        <f t="shared" si="7"/>
         <v>6.0750000000000002</v>
       </c>
       <c r="M102" t="s">
@@ -11222,11 +11222,11 @@
         <v>40000000</v>
       </c>
       <c r="K103" s="7">
-        <f>IF(OR(F103="species", F103="genus"), (I103*10^4)/J103,"NA")</f>
+        <f t="shared" si="6"/>
         <v>0.23649999999999999</v>
       </c>
       <c r="L103" s="7">
-        <f>IF(H103="percent", I103/(J103/10^6), "NA")</f>
+        <f t="shared" si="7"/>
         <v>23.65</v>
       </c>
       <c r="M103" t="s">
@@ -11269,11 +11269,11 @@
         <v>40000000</v>
       </c>
       <c r="K104" s="7">
-        <f>IF(OR(F104="species", F104="genus"), (I104*10^4)/J104,"NA")</f>
+        <f t="shared" si="6"/>
         <v>0.23749999999999999</v>
       </c>
       <c r="L104" s="7">
-        <f>IF(H104="percent", I104/(J104/10^6), "NA")</f>
+        <f t="shared" si="7"/>
         <v>23.75</v>
       </c>
       <c r="M104" t="s">
@@ -11316,11 +11316,11 @@
         <v>100000000</v>
       </c>
       <c r="K105" s="7" t="str">
-        <f>IF(OR(F105="species", F105="genus"), (I105*10^4)/J105,"NA")</f>
+        <f t="shared" si="6"/>
         <v>NA</v>
       </c>
       <c r="L105" s="7">
-        <f>IF(H105="percent", I105/(J105/10^6), "NA")</f>
+        <f t="shared" si="7"/>
         <v>6</v>
       </c>
       <c r="M105" t="s">
@@ -11363,11 +11363,11 @@
         <v>500000000</v>
       </c>
       <c r="K106" s="7" t="str">
-        <f>IF(OR(F106="species", F106="genus"), (I106*10^4)/J106,"NA")</f>
+        <f t="shared" si="6"/>
         <v>NA</v>
       </c>
       <c r="L106" s="7">
-        <f>IF(H106="percent", I106/(J106/10^6), "NA")</f>
+        <f t="shared" si="7"/>
         <v>0.91600000000000004</v>
       </c>
       <c r="M106" t="s">
@@ -11410,11 +11410,11 @@
         <v>500000000</v>
       </c>
       <c r="K107" s="7" t="str">
-        <f>IF(OR(F107="species", F107="genus"), (I107*10^4)/J107,"NA")</f>
+        <f t="shared" si="6"/>
         <v>NA</v>
       </c>
       <c r="L107" s="7">
-        <f>IF(H107="percent", I107/(J107/10^6), "NA")</f>
+        <f t="shared" si="7"/>
         <v>376</v>
       </c>
       <c r="M107" t="s">
@@ -11468,14 +11468,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d7940701-fd28-48c6-89b6-2769869457dd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11674,27 +11672,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d7940701-fd28-48c6-89b6-2769869457dd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F179CFA0-01D1-49C4-829E-9CD6990EDE07}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C242F3B7-E13F-47B3-89BF-DC7F2A584373}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="d7940701-fd28-48c6-89b6-2769869457dd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11719,9 +11710,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C242F3B7-E13F-47B3-89BF-DC7F2A584373}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F179CFA0-01D1-49C4-829E-9CD6990EDE07}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="d7940701-fd28-48c6-89b6-2769869457dd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update data for Quaternary megafaunal extinction
</commit_message>
<xml_diff>
--- a/data/disruptors_supplementary_data_tables_s1-s5.xlsx
+++ b/data/disruptors_supplementary_data_tables_s1-s5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniofleicester.sharepoint.com/sites/Team_caad90aa-a47f-449b-818d-a866be7fd445/Shared Documents/General/disruptors/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="127" documentId="14_{07CC9888-B577-4F29-BB79-BFAB3ACC8C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A116BA5-859F-4B0C-ACA3-FFDFE6D6AB2B}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="14_{07CC9888-B577-4F29-BB79-BFAB3ACC8C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFA6BB95-C7CD-444A-B6E1-FDAE491F3022}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-2895" windowWidth="29040" windowHeight="15840" firstSheet="6" activeTab="6" xr2:uid="{3126E51C-B0E9-457E-98E2-44FE6544FF4A}"/>
+    <workbookView xWindow="-28920" yWindow="-3870" windowWidth="29040" windowHeight="15840" firstSheet="6" activeTab="6" xr2:uid="{3126E51C-B0E9-457E-98E2-44FE6544FF4A}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1442" uniqueCount="710">
   <si>
     <r>
       <t>Supplementary Data tables for Wong Hearing et al.: "</t>
@@ -2175,9 +2175,6 @@
     <t>global plants</t>
   </si>
   <si>
-    <t>largely following data in Barnosky 2008</t>
-  </si>
-  <si>
     <t>global animals</t>
   </si>
   <si>
@@ -2305,6 +2302,9 @@
   </si>
   <si>
     <t>estimate of lost biomass of marine mammals and fish weighing more than 10 g over 20th century due to fishing and whaling (~2 Gt loss)</t>
+  </si>
+  <si>
+    <t>Quaternary megafaunal extinction duration and rate calculated over 50 ka to 3 ka following Bar-On et al (2018); data largely following data in Barnosky 2008</t>
   </si>
 </sst>
 </file>
@@ -2497,10 +2497,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3228,10 +3224,10 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="B44" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
@@ -7298,8 +7294,7 @@
         <v>-83</v>
       </c>
       <c r="J16" s="2">
-        <f>_xlfn.XLOOKUP(A16, table_s3_events!A:A, table_s3_events!J:J)</f>
-        <v>200</v>
+        <v>47000</v>
       </c>
       <c r="K16" s="7" t="str">
         <f t="shared" si="0"/>
@@ -7307,13 +7302,13 @@
       </c>
       <c r="L16" s="7">
         <f t="shared" si="1"/>
-        <v>-415000</v>
+        <v>-1765.9574468085107</v>
       </c>
       <c r="M16" t="s">
+        <v>709</v>
+      </c>
+      <c r="O16" t="s">
         <v>666</v>
-      </c>
-      <c r="O16" t="s">
-        <v>667</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.35">
@@ -7339,7 +7334,7 @@
         <v>637</v>
       </c>
       <c r="G17" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="H17" t="s">
         <v>634</v>
@@ -7348,19 +7343,21 @@
         <v>-50</v>
       </c>
       <c r="J17" s="2">
-        <f>_xlfn.XLOOKUP(A17, table_s3_events!A:A, table_s3_events!J:J)</f>
-        <v>200</v>
+        <v>47000</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="0"/>
-        <v>-2500</v>
+        <v>-10.638297872340425</v>
       </c>
       <c r="L17" s="7">
         <f t="shared" si="1"/>
-        <v>-250000</v>
+        <v>-1063.8297872340424</v>
+      </c>
+      <c r="M17" t="s">
+        <v>709</v>
       </c>
       <c r="O17" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.35">
@@ -7407,10 +7404,10 @@
         <v>-150000</v>
       </c>
       <c r="M18" t="s">
+        <v>669</v>
+      </c>
+      <c r="O18" t="s">
         <v>670</v>
-      </c>
-      <c r="O18" t="s">
-        <v>671</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.35">
@@ -7430,13 +7427,13 @@
         <v>0</v>
       </c>
       <c r="E19" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="F19" t="s">
         <v>646</v>
       </c>
       <c r="G19" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H19" t="s">
         <v>634</v>
@@ -7457,10 +7454,10 @@
         <v>-300000</v>
       </c>
       <c r="M19" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="O19" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.35">
@@ -7507,10 +7504,10 @@
         <v>-8050</v>
       </c>
       <c r="M20" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="O20" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.35">
@@ -7536,7 +7533,7 @@
         <v>632</v>
       </c>
       <c r="G21" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="H21" t="s">
         <v>634</v>
@@ -7557,10 +7554,10 @@
         <v>-7700</v>
       </c>
       <c r="M21" t="s">
+        <v>671</v>
+      </c>
+      <c r="O21" t="s">
         <v>672</v>
-      </c>
-      <c r="O21" t="s">
-        <v>673</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.35">
@@ -7607,10 +7604,10 @@
         <v>-4400</v>
       </c>
       <c r="M22" t="s">
+        <v>673</v>
+      </c>
+      <c r="O22" t="s">
         <v>674</v>
-      </c>
-      <c r="O22" t="s">
-        <v>675</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.35">
@@ -7636,7 +7633,7 @@
         <v>632</v>
       </c>
       <c r="G23" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H23" t="s">
         <v>634</v>
@@ -7657,10 +7654,10 @@
         <v>-2899.9999999999995</v>
       </c>
       <c r="M23" t="s">
+        <v>675</v>
+      </c>
+      <c r="O23" t="s">
         <v>676</v>
-      </c>
-      <c r="O23" t="s">
-        <v>677</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.35">
@@ -7707,7 +7704,7 @@
         <v>-2500</v>
       </c>
       <c r="O24" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.35">
@@ -7754,7 +7751,7 @@
         <v>-2250</v>
       </c>
       <c r="M25" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.35">
@@ -7801,7 +7798,7 @@
         <v>-850</v>
       </c>
       <c r="M26" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.35">
@@ -7871,7 +7868,7 @@
         <v>632</v>
       </c>
       <c r="G28" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="H28" t="s">
         <v>634</v>
@@ -7892,7 +7889,7 @@
         <v>-5000</v>
       </c>
       <c r="M28" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.35">
@@ -7939,7 +7936,7 @@
         <v>-1</v>
       </c>
       <c r="M29" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.35">
@@ -7986,7 +7983,7 @@
         <v>-22</v>
       </c>
       <c r="M30" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.35">
@@ -8012,7 +8009,7 @@
         <v>632</v>
       </c>
       <c r="G31" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="H31" t="s">
         <v>634</v>
@@ -8033,7 +8030,7 @@
         <v>-72</v>
       </c>
       <c r="M31" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.35">
@@ -8059,7 +8056,7 @@
         <v>637</v>
       </c>
       <c r="G32" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="H32" t="s">
         <v>634</v>
@@ -8080,7 +8077,7 @@
         <v>-98</v>
       </c>
       <c r="M32" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.35">
@@ -8106,7 +8103,7 @@
         <v>637</v>
       </c>
       <c r="G33" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="H33" t="s">
         <v>634</v>
@@ -8127,7 +8124,7 @@
         <v>-84</v>
       </c>
       <c r="M33" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.35">
@@ -8614,7 +8611,7 @@
         <v>-2500000</v>
       </c>
       <c r="M44" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.35">
@@ -8749,7 +8746,7 @@
         <v>2</v>
       </c>
       <c r="M47" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.35">
@@ -8796,7 +8793,7 @@
         <v>2.1466666666666665</v>
       </c>
       <c r="M48" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.35">
@@ -9238,7 +9235,7 @@
         <v>-56.880733944954123</v>
       </c>
       <c r="M58" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.35">
@@ -9285,7 +9282,7 @@
         <v>-46.788990825688067</v>
       </c>
       <c r="M59" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.35">
@@ -9332,7 +9329,7 @@
         <v>-30.275229357798164</v>
       </c>
       <c r="M60" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.35">
@@ -10617,7 +10614,7 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="M89" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.35">
@@ -10664,7 +10661,7 @@
         <v>1.3333333333333333</v>
       </c>
       <c r="M90" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.35">
@@ -10711,7 +10708,7 @@
         <v>2.4500000000000002</v>
       </c>
       <c r="M91" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.35">
@@ -10758,7 +10755,7 @@
         <v>15</v>
       </c>
       <c r="M92" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.35">
@@ -10805,7 +10802,7 @@
         <v>200</v>
       </c>
       <c r="M93" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.35">
@@ -10852,7 +10849,7 @@
         <v>300</v>
       </c>
       <c r="M94" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.35">
@@ -10898,7 +10895,7 @@
         <v>26.666666666666668</v>
       </c>
       <c r="M95" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.35">
@@ -10989,7 +10986,7 @@
         <v>-23.076923076923077</v>
       </c>
       <c r="M97" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="98" spans="1:13" x14ac:dyDescent="0.35">
@@ -11124,7 +11121,7 @@
         <v>-100</v>
       </c>
       <c r="M100" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="101" spans="1:13" x14ac:dyDescent="0.35">
@@ -11171,7 +11168,7 @@
         <v>-50</v>
       </c>
       <c r="M101" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="102" spans="1:13" x14ac:dyDescent="0.35">
@@ -11262,7 +11259,7 @@
         <v>6.0750000000000002</v>
       </c>
       <c r="M103" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.35">
@@ -11288,7 +11285,7 @@
         <v>637</v>
       </c>
       <c r="G104" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H104" t="s">
         <v>634</v>
@@ -11309,7 +11306,7 @@
         <v>23.65</v>
       </c>
       <c r="M104" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.35">
@@ -11335,7 +11332,7 @@
         <v>632</v>
       </c>
       <c r="G105" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H105" t="s">
         <v>634</v>
@@ -11356,7 +11353,7 @@
         <v>23.75</v>
       </c>
       <c r="M105" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="106" spans="1:13" x14ac:dyDescent="0.35">
@@ -11403,7 +11400,7 @@
         <v>6</v>
       </c>
       <c r="M106" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.35">
@@ -11450,7 +11447,7 @@
         <v>0.91600000000000004</v>
       </c>
       <c r="M107" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.35">
@@ -11497,7 +11494,7 @@
         <v>376</v>
       </c>
       <c r="M108" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
     </row>
   </sheetData>
@@ -11556,6 +11553,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d7940701-fd28-48c6-89b6-2769869457dd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EE3B5FF1D6D93545B0A9BE76E04A5739" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b213452e5774ccb18cdbac914376359f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af" xmlns:ns3="d7940701-fd28-48c6-89b6-2769869457dd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="94bb0651eba29840b02d7d9879aff2b0" ns2:_="" ns3:_="">
     <xsd:import namespace="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
@@ -11750,17 +11758,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d7940701-fd28-48c6-89b6-2769869457dd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C242F3B7-E13F-47B3-89BF-DC7F2A584373}">
   <ds:schemaRefs>
@@ -11770,6 +11767,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F179CFA0-01D1-49C4-829E-9CD6990EDE07}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d7940701-fd28-48c6-89b6-2769869457dd"/>
+    <ds:schemaRef ds:uri="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14D4D638-0E0C-48CA-BE88-3BE2B56E957A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11786,15 +11794,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F179CFA0-01D1-49C4-829E-9CD6990EDE07}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d7940701-fd28-48c6-89b6-2769869457dd"/>
-    <ds:schemaRef ds:uri="f4d1a5f8-cfe9-4a60-92ce-29fb37cf63af"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>